<commit_message>
data: publish 2026-10-29 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-29-182路.xlsx
+++ b/data/export/2026-10-29-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC9"/>
+  <dimension ref="A1:AC15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -715,7 +715,7 @@
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA3" s="2" t="inlineStr">
@@ -826,7 +826,7 @@
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>06:32</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -937,7 +937,7 @@
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>06:42</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1159,7 +1159,7 @@
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>06:52</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1270,7 +1270,7 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>06:52</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1381,7 +1381,7 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -1389,22 +1389,22 @@
       <c r="A9" s="2" t="inlineStr"/>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>沪A32298D</t>
+          <t>沪A35717D</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>07:25</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1437,12 +1437,12 @@
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:42</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>07:25</t>
+          <t>07:12</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
@@ -1492,7 +1492,673 @@
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>06:52</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A32298D</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>07:25</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:25</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A02126A</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-10-29 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-29-182路.xlsx
+++ b/data/export/2026-10-29-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC28"/>
+  <dimension ref="A1:AC31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -665,7 +665,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>07:52</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>09:22</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>08:12</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>09:22</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>08:33</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr">
@@ -1775,7 +1775,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>09:22</t>
+          <t>09:32</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>09:22</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>09:22</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>07:52</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="Z15" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA15" s="2" t="inlineStr">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>08:12</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="Z16" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA16" s="2" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>09:22</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>08:33</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="Z19" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA19" s="2" t="inlineStr">
@@ -3218,7 +3218,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>09:22</t>
+          <t>09:32</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>09:22</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -3440,7 +3440,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>09:22</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -3498,22 +3498,22 @@
       <c r="A28" s="2" t="inlineStr"/>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>沪A67026D</t>
+          <t>沪A67983D</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
           <t>川沙客运站</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>10:15</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>金杨路金口路</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>09:22</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -3565,7 +3565,7 @@
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>10:05</t>
         </is>
       </c>
       <c r="V28" s="2" t="inlineStr">
@@ -3600,6 +3600,339 @@
       </c>
       <c r="AB28" s="2" t="inlineStr"/>
       <c r="AC28" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>09:42</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="inlineStr"/>
+      <c r="R29" s="2" t="inlineStr"/>
+      <c r="S29" s="2" t="inlineStr"/>
+      <c r="T29" s="2" t="inlineStr"/>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="V29" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W29" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X29" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y29" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z29" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA29" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB29" s="2" t="inlineStr"/>
+      <c r="AC29" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>沪A13735A</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>09:42</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr"/>
+      <c r="R30" s="2" t="inlineStr"/>
+      <c r="S30" s="2" t="inlineStr"/>
+      <c r="T30" s="2" t="inlineStr"/>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="V30" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W30" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y30" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z30" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA30" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB30" s="2" t="inlineStr"/>
+      <c r="AC30" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr"/>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>沪A66513D</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr"/>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>09:42</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q31" s="2" t="inlineStr"/>
+      <c r="R31" s="2" t="inlineStr"/>
+      <c r="S31" s="2" t="inlineStr"/>
+      <c r="T31" s="2" t="inlineStr"/>
+      <c r="U31" s="2" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="V31" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W31" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X31" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y31" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z31" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA31" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB31" s="2" t="inlineStr"/>
+      <c r="AC31" s="2" t="inlineStr">
         <is>
           <t>—/13</t>
         </is>

</xml_diff>